<commit_message>
Fixes catalogo y login
</commit_message>
<xml_diff>
--- a/data/inventario.xlsx
+++ b/data/inventario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Trabajos\Riviere\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C63ED969-D6A9-46B5-9A78-73BE9DB1B319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A7858C-F2B4-40BE-B325-FBCDE582C829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventario" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Inventario!$A$1:$I$136</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="151">
   <si>
     <t>Estilo</t>
   </si>
@@ -2014,11 +2015,11 @@
       <c r="A37" t="s">
         <v>56</v>
       </c>
-      <c r="C37" t="s">
-        <v>57</v>
+      <c r="C37">
+        <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="E37" t="s">
         <v>58</v>

</xml_diff>